<commit_message>
Improve extraction accuracy and stability, update template
- Tighten prompt rules for product_name (no AI-added descriptive words)
  and size_range (prefer order-specific/measurement-spec sizes over
  abbreviated cover-page size labels)
- Normalize embedded newlines when flattening Excel cells to text so
  size rows aren't visually split and truncated
- Add local result cache keyed by file content hash so re-extracting
  the same tech pack returns identical output instead of re-querying
  the model
- Update excel_writer image placement/sizing and add plain-text
  flattening safeguard for cell values
- Update template to drop AI-marker highlighting
- Remove stray committed .pyc, add .gitignore
</commit_message>
<xml_diff>
--- a/templates/报价单总表模板.xlsx
+++ b/templates/报价单总表模板.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="11620" tabRatio="595"/>
+    <workbookView windowWidth="24420" windowHeight="12600" tabRatio="595"/>
   </bookViews>
   <sheets>
     <sheet name="总表-高亮黄色需要AI介入" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="151">
   <si>
     <r>
       <rPr>
@@ -274,62 +274,10 @@
     <t>工厂回复</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>面料品质</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>--</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>正染</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>面料颜色</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>印花</t>
-    </r>
+    <t>面料品质--正染</t>
+  </si>
+  <si>
+    <t>面料颜色/印花</t>
   </si>
   <si>
     <t>数量</t>
@@ -356,147 +304,8 @@
     <t>报价情况</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>FOB</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>柬埔寨</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>含税（增值税发票</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>+</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>物流发票）含运费</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>，入</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>6</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>个仓库</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>不需要</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>AI</t>
-    </r>
-  </si>
-  <si>
-    <t>需要AI在客人资料中提取</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>需要</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <charset val="0"/>
-      </rPr>
-      <t>AI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="宋体"/>
-        <charset val="0"/>
-      </rPr>
-      <t>在订单资料中提取</t>
-    </r>
-  </si>
-  <si>
-    <t>需要AI在客人资料中提取，且翻译</t>
+    <t>FOB柬埔寨
+含税（增值税发票+物流发票）含运费 ，入6个仓库</t>
   </si>
   <si>
     <r>
@@ -3701,7 +3510,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.0_ "/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="34">
     <font>
       <sz val="12"/>
       <name val="宋体"/>
@@ -3746,11 +3555,6 @@
       <charset val="0"/>
     </font>
     <font>
-      <sz val="14"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
@@ -3768,12 +3572,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="14"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -3905,6 +3703,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="宋体"/>
       <charset val="0"/>
     </font>
@@ -4275,154 +4079,154 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4516,10 +4320,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
@@ -4537,61 +4341,49 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="1" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="1" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
@@ -6768,8 +6560,8 @@
       <c r="P1" s="37"/>
       <c r="Q1" s="37"/>
       <c r="R1" s="37"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="50"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="47"/>
     </row>
     <row r="2" ht="56" customHeight="1" spans="1:20">
       <c r="A2" s="38" t="s">
@@ -6792,8 +6584,8 @@
       <c r="P2" s="38"/>
       <c r="Q2" s="38"/>
       <c r="R2" s="38"/>
-      <c r="S2" s="51"/>
-      <c r="T2" s="52"/>
+      <c r="S2" s="48"/>
+      <c r="T2" s="49"/>
     </row>
     <row r="3" ht="56" customHeight="1" spans="1:20">
       <c r="A3" s="39" t="s">
@@ -6808,7 +6600,7 @@
       <c r="H3" s="40"/>
       <c r="I3" s="40"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="48"/>
+      <c r="K3" s="46"/>
       <c r="L3" s="40"/>
       <c r="M3" s="40"/>
       <c r="N3" s="40"/>
@@ -6816,50 +6608,50 @@
       <c r="P3" s="40"/>
       <c r="Q3" s="40"/>
       <c r="R3" s="40"/>
-      <c r="S3" s="48"/>
-      <c r="T3" s="53"/>
-    </row>
-    <row r="4" customHeight="1" spans="1:20">
+      <c r="S3" s="46"/>
+      <c r="T3" s="50"/>
+    </row>
+    <row r="4" ht="56" customHeight="1" spans="1:20">
       <c r="A4" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="47" t="s">
+      <c r="G4" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="41" t="s">
+      <c r="H4" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="41" t="s">
+      <c r="I4" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="47" t="s">
+      <c r="J4" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="41" t="s">
+      <c r="L4" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="41" t="s">
+      <c r="M4" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="41" t="s">
+      <c r="N4" s="42" t="s">
         <v>15</v>
       </c>
       <c r="O4" s="41" t="s">
@@ -6871,77 +6663,36 @@
       <c r="Q4" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="R4" s="54" t="s">
+      <c r="R4" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="S4" s="54" t="s">
+      <c r="S4" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="T4" s="55" t="s">
+      <c r="T4" s="52" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" s="30" customFormat="1" customHeight="1" spans="1:20">
-      <c r="A5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="43" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="K5" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="L5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="M5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="N5" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="O5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="P5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="R5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="S5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="T5" s="42" t="s">
-        <v>22</v>
-      </c>
+      <c r="A5" s="42"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
+      <c r="L5" s="43"/>
+      <c r="M5" s="43"/>
+      <c r="O5" s="42"/>
+      <c r="P5" s="42"/>
+      <c r="Q5" s="42"/>
+      <c r="R5" s="42"/>
+      <c r="S5" s="42"/>
+      <c r="T5" s="42"/>
     </row>
     <row r="6" s="31" customFormat="1" customHeight="1" spans="1:20">
       <c r="A6" s="44"/>
@@ -6966,26 +6717,26 @@
       <c r="T6" s="44"/>
     </row>
     <row r="7" s="32" customFormat="1" customHeight="1" spans="1:20">
-      <c r="A7" s="45"/>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
-      <c r="O7" s="45"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="45"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
+      <c r="N7" s="44"/>
+      <c r="O7" s="44"/>
+      <c r="P7" s="44"/>
+      <c r="Q7" s="44"/>
+      <c r="R7" s="44"/>
+      <c r="S7" s="44"/>
+      <c r="T7" s="44"/>
     </row>
     <row r="8" s="31" customFormat="1" customHeight="1" spans="1:20">
       <c r="A8" s="44"/>
@@ -7010,444 +6761,444 @@
       <c r="T8" s="44"/>
     </row>
     <row r="9" customHeight="1" spans="1:20">
-      <c r="A9" s="46"/>
-      <c r="B9" s="46"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
-      <c r="J9" s="46"/>
-      <c r="K9" s="46"/>
-      <c r="L9" s="46"/>
-      <c r="M9" s="46"/>
-      <c r="N9" s="46"/>
-      <c r="O9" s="46"/>
-      <c r="P9" s="46"/>
-      <c r="Q9" s="46"/>
-      <c r="R9" s="46"/>
-      <c r="S9" s="46"/>
-      <c r="T9" s="46"/>
+      <c r="A9" s="45"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+      <c r="O9" s="45"/>
+      <c r="P9" s="45"/>
+      <c r="Q9" s="45"/>
+      <c r="R9" s="45"/>
+      <c r="S9" s="45"/>
+      <c r="T9" s="45"/>
     </row>
     <row r="10" customHeight="1" spans="1:20">
-      <c r="A10" s="46"/>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="49"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
-      <c r="N10" s="46"/>
-      <c r="O10" s="46"/>
-      <c r="P10" s="46"/>
-      <c r="Q10" s="46"/>
-      <c r="R10" s="46"/>
-      <c r="S10" s="56"/>
-      <c r="T10" s="57"/>
+      <c r="A10" s="45"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="37"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="45"/>
+      <c r="O10" s="45"/>
+      <c r="P10" s="45"/>
+      <c r="Q10" s="45"/>
+      <c r="R10" s="45"/>
+      <c r="S10" s="46"/>
+      <c r="T10" s="53"/>
     </row>
     <row r="11" customHeight="1" spans="1:20">
-      <c r="A11" s="46"/>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="46"/>
-      <c r="K11" s="49"/>
-      <c r="L11" s="46"/>
-      <c r="M11" s="46"/>
-      <c r="N11" s="46"/>
-      <c r="O11" s="46"/>
-      <c r="P11" s="46"/>
-      <c r="Q11" s="46"/>
-      <c r="R11" s="46"/>
-      <c r="S11" s="56"/>
-      <c r="T11" s="57"/>
+      <c r="A11" s="45"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="45"/>
+      <c r="Q11" s="45"/>
+      <c r="R11" s="45"/>
+      <c r="S11" s="46"/>
+      <c r="T11" s="53"/>
     </row>
     <row r="12" customHeight="1" spans="1:20">
-      <c r="A12" s="46"/>
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="46"/>
-      <c r="K12" s="49"/>
-      <c r="L12" s="46"/>
-      <c r="M12" s="46"/>
-      <c r="N12" s="46"/>
-      <c r="O12" s="46"/>
-      <c r="P12" s="46"/>
-      <c r="Q12" s="46"/>
-      <c r="R12" s="46"/>
-      <c r="S12" s="56"/>
-      <c r="T12" s="57"/>
+      <c r="A12" s="45"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="45"/>
+      <c r="M12" s="45"/>
+      <c r="N12" s="45"/>
+      <c r="O12" s="45"/>
+      <c r="P12" s="45"/>
+      <c r="Q12" s="45"/>
+      <c r="R12" s="45"/>
+      <c r="S12" s="46"/>
+      <c r="T12" s="53"/>
     </row>
     <row r="13" customHeight="1" spans="1:20">
-      <c r="A13" s="46"/>
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="46"/>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46"/>
-      <c r="H13" s="46"/>
-      <c r="I13" s="46"/>
-      <c r="J13" s="46"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="46"/>
-      <c r="M13" s="46"/>
-      <c r="N13" s="46"/>
-      <c r="O13" s="46"/>
-      <c r="P13" s="46"/>
-      <c r="Q13" s="46"/>
-      <c r="R13" s="46"/>
-      <c r="S13" s="56"/>
-      <c r="T13" s="57"/>
+      <c r="A13" s="45"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="45"/>
+      <c r="M13" s="45"/>
+      <c r="N13" s="45"/>
+      <c r="O13" s="45"/>
+      <c r="P13" s="45"/>
+      <c r="Q13" s="45"/>
+      <c r="R13" s="45"/>
+      <c r="S13" s="46"/>
+      <c r="T13" s="53"/>
     </row>
     <row r="14" customHeight="1" spans="1:20">
-      <c r="A14" s="46"/>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="49"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
-      <c r="N14" s="46"/>
-      <c r="O14" s="46"/>
-      <c r="P14" s="46"/>
-      <c r="Q14" s="46"/>
-      <c r="R14" s="46"/>
-      <c r="S14" s="56"/>
-      <c r="T14" s="57"/>
+      <c r="A14" s="45"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="37"/>
+      <c r="L14" s="45"/>
+      <c r="M14" s="45"/>
+      <c r="N14" s="45"/>
+      <c r="O14" s="45"/>
+      <c r="P14" s="45"/>
+      <c r="Q14" s="45"/>
+      <c r="R14" s="45"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="53"/>
     </row>
     <row r="15" customHeight="1" spans="1:20">
-      <c r="A15" s="46"/>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="46"/>
-      <c r="K15" s="49"/>
-      <c r="L15" s="46"/>
-      <c r="M15" s="46"/>
-      <c r="N15" s="46"/>
-      <c r="O15" s="46"/>
-      <c r="P15" s="46"/>
-      <c r="Q15" s="46"/>
-      <c r="R15" s="46"/>
-      <c r="S15" s="56"/>
-      <c r="T15" s="57"/>
+      <c r="A15" s="45"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
+      <c r="O15" s="45"/>
+      <c r="P15" s="45"/>
+      <c r="Q15" s="45"/>
+      <c r="R15" s="45"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="53"/>
     </row>
     <row r="16" customHeight="1" spans="1:20">
-      <c r="A16" s="46"/>
-      <c r="B16" s="46"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="46"/>
-      <c r="K16" s="49"/>
-      <c r="L16" s="46"/>
-      <c r="M16" s="46"/>
-      <c r="N16" s="46"/>
-      <c r="O16" s="46"/>
-      <c r="P16" s="46"/>
-      <c r="Q16" s="46"/>
-      <c r="R16" s="46"/>
-      <c r="S16" s="56"/>
-      <c r="T16" s="57"/>
+      <c r="A16" s="45"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="37"/>
+      <c r="L16" s="45"/>
+      <c r="M16" s="45"/>
+      <c r="N16" s="45"/>
+      <c r="O16" s="45"/>
+      <c r="P16" s="45"/>
+      <c r="Q16" s="45"/>
+      <c r="R16" s="45"/>
+      <c r="S16" s="46"/>
+      <c r="T16" s="53"/>
     </row>
     <row r="17" customHeight="1" spans="1:20">
-      <c r="A17" s="46"/>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="46"/>
-      <c r="K17" s="49"/>
-      <c r="L17" s="46"/>
-      <c r="M17" s="46"/>
-      <c r="N17" s="46"/>
-      <c r="O17" s="46"/>
-      <c r="P17" s="46"/>
-      <c r="Q17" s="46"/>
-      <c r="R17" s="46"/>
-      <c r="S17" s="56"/>
-      <c r="T17" s="57"/>
+      <c r="A17" s="45"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="45"/>
+      <c r="O17" s="45"/>
+      <c r="P17" s="45"/>
+      <c r="Q17" s="45"/>
+      <c r="R17" s="45"/>
+      <c r="S17" s="46"/>
+      <c r="T17" s="53"/>
     </row>
     <row r="18" customHeight="1" spans="1:20">
-      <c r="A18" s="46"/>
-      <c r="B18" s="46"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="46"/>
-      <c r="K18" s="49"/>
-      <c r="L18" s="46"/>
-      <c r="M18" s="46"/>
-      <c r="N18" s="46"/>
-      <c r="O18" s="46"/>
-      <c r="P18" s="46"/>
-      <c r="Q18" s="46"/>
-      <c r="R18" s="46"/>
-      <c r="S18" s="56"/>
-      <c r="T18" s="57"/>
+      <c r="A18" s="45"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="45"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="45"/>
+      <c r="O18" s="45"/>
+      <c r="P18" s="45"/>
+      <c r="Q18" s="45"/>
+      <c r="R18" s="45"/>
+      <c r="S18" s="46"/>
+      <c r="T18" s="53"/>
     </row>
     <row r="19" customHeight="1" spans="1:20">
-      <c r="A19" s="46"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="46"/>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="46"/>
-      <c r="I19" s="46"/>
-      <c r="J19" s="46"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="46"/>
-      <c r="M19" s="46"/>
-      <c r="N19" s="46"/>
-      <c r="O19" s="46"/>
-      <c r="P19" s="46"/>
-      <c r="Q19" s="46"/>
-      <c r="R19" s="46"/>
-      <c r="S19" s="56"/>
-      <c r="T19" s="57"/>
+      <c r="A19" s="45"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="45"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="45"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="45"/>
+      <c r="M19" s="45"/>
+      <c r="N19" s="45"/>
+      <c r="O19" s="45"/>
+      <c r="P19" s="45"/>
+      <c r="Q19" s="45"/>
+      <c r="R19" s="45"/>
+      <c r="S19" s="46"/>
+      <c r="T19" s="53"/>
     </row>
     <row r="20" customHeight="1" spans="1:20">
-      <c r="A20" s="46"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="46"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="46"/>
-      <c r="N20" s="46"/>
-      <c r="O20" s="46"/>
-      <c r="P20" s="46"/>
-      <c r="Q20" s="46"/>
-      <c r="R20" s="46"/>
-      <c r="S20" s="56"/>
-      <c r="T20" s="57"/>
+      <c r="A20" s="45"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="45"/>
+      <c r="M20" s="45"/>
+      <c r="N20" s="45"/>
+      <c r="O20" s="45"/>
+      <c r="P20" s="45"/>
+      <c r="Q20" s="45"/>
+      <c r="R20" s="45"/>
+      <c r="S20" s="46"/>
+      <c r="T20" s="53"/>
     </row>
     <row r="21" customHeight="1" spans="1:20">
-      <c r="A21" s="46"/>
-      <c r="B21" s="46"/>
-      <c r="C21" s="46"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46"/>
-      <c r="H21" s="46"/>
-      <c r="I21" s="46"/>
-      <c r="J21" s="46"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="46"/>
-      <c r="M21" s="46"/>
-      <c r="N21" s="46"/>
-      <c r="O21" s="46"/>
-      <c r="P21" s="46"/>
-      <c r="Q21" s="46"/>
-      <c r="R21" s="46"/>
-      <c r="S21" s="56"/>
-      <c r="T21" s="57"/>
+      <c r="A21" s="45"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="45"/>
+      <c r="G21" s="45"/>
+      <c r="H21" s="45"/>
+      <c r="I21" s="45"/>
+      <c r="J21" s="45"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="45"/>
+      <c r="M21" s="45"/>
+      <c r="N21" s="45"/>
+      <c r="O21" s="45"/>
+      <c r="P21" s="45"/>
+      <c r="Q21" s="45"/>
+      <c r="R21" s="45"/>
+      <c r="S21" s="46"/>
+      <c r="T21" s="53"/>
     </row>
     <row r="22" customHeight="1" spans="1:20">
-      <c r="A22" s="46"/>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="46"/>
-      <c r="N22" s="46"/>
-      <c r="O22" s="46"/>
-      <c r="P22" s="46"/>
-      <c r="Q22" s="46"/>
-      <c r="R22" s="46"/>
-      <c r="S22" s="56"/>
-      <c r="T22" s="57"/>
+      <c r="A22" s="45"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="45"/>
+      <c r="J22" s="45"/>
+      <c r="K22" s="37"/>
+      <c r="L22" s="45"/>
+      <c r="M22" s="45"/>
+      <c r="N22" s="45"/>
+      <c r="O22" s="45"/>
+      <c r="P22" s="45"/>
+      <c r="Q22" s="45"/>
+      <c r="R22" s="45"/>
+      <c r="S22" s="46"/>
+      <c r="T22" s="53"/>
     </row>
     <row r="23" customHeight="1" spans="1:20">
-      <c r="A23" s="46"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="46"/>
-      <c r="M23" s="46"/>
-      <c r="N23" s="46"/>
-      <c r="O23" s="46"/>
-      <c r="P23" s="46"/>
-      <c r="Q23" s="46"/>
-      <c r="R23" s="46"/>
-      <c r="S23" s="56"/>
-      <c r="T23" s="57"/>
+      <c r="A23" s="45"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="45"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="45"/>
+      <c r="M23" s="45"/>
+      <c r="N23" s="45"/>
+      <c r="O23" s="45"/>
+      <c r="P23" s="45"/>
+      <c r="Q23" s="45"/>
+      <c r="R23" s="45"/>
+      <c r="S23" s="46"/>
+      <c r="T23" s="53"/>
     </row>
     <row r="24" customHeight="1" spans="1:20">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="46"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="46"/>
-      <c r="N24" s="46"/>
-      <c r="O24" s="46"/>
-      <c r="P24" s="46"/>
-      <c r="Q24" s="46"/>
-      <c r="R24" s="46"/>
-      <c r="S24" s="56"/>
-      <c r="T24" s="57"/>
+      <c r="A24" s="45"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="45"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="45"/>
+      <c r="M24" s="45"/>
+      <c r="N24" s="45"/>
+      <c r="O24" s="45"/>
+      <c r="P24" s="45"/>
+      <c r="Q24" s="45"/>
+      <c r="R24" s="45"/>
+      <c r="S24" s="46"/>
+      <c r="T24" s="53"/>
     </row>
     <row r="25" customHeight="1" spans="1:20">
-      <c r="A25" s="46"/>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="46"/>
-      <c r="K25" s="49"/>
-      <c r="L25" s="46"/>
-      <c r="M25" s="46"/>
-      <c r="N25" s="46"/>
-      <c r="O25" s="46"/>
-      <c r="P25" s="46"/>
-      <c r="Q25" s="46"/>
-      <c r="R25" s="46"/>
-      <c r="S25" s="56"/>
-      <c r="T25" s="57"/>
+      <c r="A25" s="45"/>
+      <c r="B25" s="45"/>
+      <c r="C25" s="45"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="45"/>
+      <c r="I25" s="45"/>
+      <c r="J25" s="45"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="45"/>
+      <c r="M25" s="45"/>
+      <c r="N25" s="45"/>
+      <c r="O25" s="45"/>
+      <c r="P25" s="45"/>
+      <c r="Q25" s="45"/>
+      <c r="R25" s="45"/>
+      <c r="S25" s="46"/>
+      <c r="T25" s="53"/>
     </row>
     <row r="26" customHeight="1" spans="1:20">
-      <c r="A26" s="46"/>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="46"/>
-      <c r="H26" s="46"/>
-      <c r="I26" s="46"/>
-      <c r="J26" s="46"/>
-      <c r="K26" s="49"/>
-      <c r="L26" s="46"/>
-      <c r="M26" s="46"/>
-      <c r="N26" s="46"/>
-      <c r="O26" s="46"/>
-      <c r="P26" s="46"/>
-      <c r="Q26" s="46"/>
-      <c r="R26" s="46"/>
-      <c r="S26" s="56"/>
-      <c r="T26" s="57"/>
+      <c r="A26" s="45"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="45"/>
+      <c r="J26" s="45"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="45"/>
+      <c r="M26" s="45"/>
+      <c r="N26" s="45"/>
+      <c r="O26" s="45"/>
+      <c r="P26" s="45"/>
+      <c r="Q26" s="45"/>
+      <c r="R26" s="45"/>
+      <c r="S26" s="46"/>
+      <c r="T26" s="53"/>
     </row>
     <row r="27" customHeight="1" spans="1:20">
-      <c r="A27" s="46"/>
-      <c r="B27" s="46"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="46"/>
-      <c r="F27" s="46"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="46"/>
-      <c r="I27" s="46"/>
-      <c r="J27" s="46"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="46"/>
-      <c r="M27" s="46"/>
-      <c r="N27" s="46"/>
-      <c r="O27" s="46"/>
-      <c r="P27" s="46"/>
-      <c r="Q27" s="46"/>
-      <c r="R27" s="46"/>
-      <c r="S27" s="56"/>
-      <c r="T27" s="57"/>
+      <c r="A27" s="45"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="45"/>
+      <c r="J27" s="45"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="45"/>
+      <c r="M27" s="45"/>
+      <c r="N27" s="45"/>
+      <c r="O27" s="45"/>
+      <c r="P27" s="45"/>
+      <c r="Q27" s="45"/>
+      <c r="R27" s="45"/>
+      <c r="S27" s="46"/>
+      <c r="T27" s="53"/>
     </row>
     <row r="28" customHeight="1" spans="1:20">
-      <c r="A28" s="46"/>
-      <c r="B28" s="46"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="46"/>
-      <c r="H28" s="46"/>
-      <c r="I28" s="46"/>
-      <c r="J28" s="46"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="46"/>
-      <c r="M28" s="46"/>
-      <c r="N28" s="46"/>
-      <c r="O28" s="46"/>
-      <c r="P28" s="46"/>
-      <c r="Q28" s="46"/>
-      <c r="R28" s="46"/>
-      <c r="S28" s="56"/>
-      <c r="T28" s="57"/>
+      <c r="A28" s="45"/>
+      <c r="B28" s="45"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="45"/>
+      <c r="H28" s="45"/>
+      <c r="I28" s="45"/>
+      <c r="J28" s="45"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="45"/>
+      <c r="M28" s="45"/>
+      <c r="N28" s="45"/>
+      <c r="O28" s="45"/>
+      <c r="P28" s="45"/>
+      <c r="Q28" s="45"/>
+      <c r="R28" s="45"/>
+      <c r="S28" s="46"/>
+      <c r="T28" s="53"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:U8" etc:filterBottomFollowUsedRange="0">
@@ -7493,311 +7244,311 @@
     </row>
     <row r="2" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I2" s="6"/>
     </row>
     <row r="3" s="20" customFormat="1" ht="51" customHeight="1" spans="1:9">
       <c r="A3" s="2"/>
       <c r="B3" s="9" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
       <c r="H3" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I3" s="9"/>
     </row>
     <row r="4" s="20" customFormat="1" ht="51" hidden="1" customHeight="1" spans="1:9">
       <c r="A4" s="2"/>
       <c r="B4" s="17" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C4" s="18"/>
       <c r="D4" s="22" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
       <c r="G4" s="26"/>
       <c r="H4" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I4" s="9"/>
     </row>
     <row r="5" s="20" customFormat="1" ht="51" customHeight="1" spans="1:9">
       <c r="A5" s="2"/>
       <c r="B5" s="9" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
       <c r="H5" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I5" s="9"/>
     </row>
     <row r="6" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A6" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I6" s="6"/>
     </row>
     <row r="7" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A7" s="6"/>
       <c r="B7" s="9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
       <c r="H7" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I7" s="9"/>
     </row>
     <row r="8" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A8" s="6"/>
       <c r="B8" s="9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I8" s="9"/>
     </row>
     <row r="9" s="20" customFormat="1" ht="60.95" hidden="1" customHeight="1" spans="1:9">
       <c r="A9" s="6"/>
       <c r="B9" s="17" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="22" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E9" s="25"/>
       <c r="F9" s="25"/>
       <c r="G9" s="26"/>
       <c r="H9" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I9" s="9"/>
     </row>
     <row r="10" s="21" customFormat="1" ht="57.95" hidden="1" customHeight="1" spans="1:9">
       <c r="A10" s="6"/>
       <c r="B10" s="17" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C10" s="18"/>
       <c r="D10" s="17" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="27"/>
       <c r="G10" s="18"/>
       <c r="H10" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I10" s="9"/>
     </row>
     <row r="11" s="21" customFormat="1" ht="36.95" customHeight="1" spans="1:9">
       <c r="A11" s="6"/>
       <c r="B11" s="17" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C11" s="18"/>
       <c r="D11" s="23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
       <c r="G11" s="29"/>
       <c r="H11" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I11" s="9"/>
     </row>
     <row r="12" s="21" customFormat="1" ht="60.95" customHeight="1" spans="1:9">
       <c r="A12" s="6"/>
       <c r="B12" s="17" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C12" s="18"/>
       <c r="D12" s="17" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="27"/>
       <c r="G12" s="18"/>
       <c r="H12" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I12" s="9"/>
     </row>
     <row r="13" s="21" customFormat="1" ht="42" hidden="1" customHeight="1" spans="1:9">
       <c r="A13" s="6"/>
       <c r="B13" s="17" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C13" s="18"/>
       <c r="D13" s="17" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E13" s="27"/>
       <c r="F13" s="27"/>
       <c r="G13" s="18"/>
       <c r="H13" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I13" s="9"/>
     </row>
     <row r="14" s="21" customFormat="1" ht="39" customHeight="1" spans="1:9">
       <c r="A14" s="6"/>
       <c r="B14" s="17" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27"/>
       <c r="G14" s="18"/>
       <c r="H14" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I14" s="9"/>
     </row>
     <row r="15" s="21" customFormat="1" ht="33" customHeight="1" spans="1:9">
       <c r="A15" s="6"/>
       <c r="B15" s="17" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="27"/>
       <c r="G15" s="18"/>
       <c r="H15" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I15" s="9"/>
     </row>
     <row r="16" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A16" s="24"/>
       <c r="B16" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I16" s="9"/>
     </row>
     <row r="17" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A17" s="24"/>
       <c r="B17" s="9" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I17" s="9"/>
     </row>
     <row r="18" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A18" s="24"/>
       <c r="B18" s="9" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I18" s="9"/>
     </row>
     <row r="19" s="20" customFormat="1" ht="36" customHeight="1" spans="1:9">
       <c r="A19" s="24"/>
       <c r="B19" s="9" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I19" s="9"/>
     </row>
@@ -7895,7 +7646,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="17" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7905,24 +7656,24 @@
     </row>
     <row r="2" s="1" customFormat="1" ht="81" customHeight="1" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:6">
       <c r="A3" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
       <c r="D3" s="4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
@@ -7932,26 +7683,26 @@
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
     </row>
     <row r="5" s="1" customFormat="1" ht="17" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
       <c r="D5" s="7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
     </row>
     <row r="6" s="1" customFormat="1" spans="1:6">
       <c r="A6" s="5" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -7961,17 +7712,17 @@
     </row>
     <row r="7" s="1" customFormat="1" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -7979,11 +7730,11 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F8" s="9"/>
     </row>
@@ -7991,11 +7742,11 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F9" s="9"/>
     </row>
@@ -8003,11 +7754,11 @@
       <c r="A10" s="6"/>
       <c r="B10" s="2"/>
       <c r="C10" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F10" s="9"/>
     </row>
@@ -8015,11 +7766,11 @@
       <c r="A11" s="6"/>
       <c r="B11" s="2"/>
       <c r="C11" s="8" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F11" s="6"/>
     </row>
@@ -8027,11 +7778,11 @@
       <c r="A12" s="6"/>
       <c r="B12" s="2"/>
       <c r="C12" s="8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F12" s="9"/>
     </row>
@@ -8039,11 +7790,11 @@
       <c r="A13" s="6"/>
       <c r="B13" s="2"/>
       <c r="C13" s="8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F13" s="9"/>
     </row>
@@ -8051,11 +7802,11 @@
       <c r="A14" s="6"/>
       <c r="B14" s="2"/>
       <c r="C14" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F14" s="9"/>
     </row>
@@ -8063,11 +7814,11 @@
       <c r="A15" s="6"/>
       <c r="B15" s="2"/>
       <c r="C15" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F15" s="9"/>
     </row>
@@ -8075,11 +7826,11 @@
       <c r="A16" s="6"/>
       <c r="B16" s="2"/>
       <c r="C16" s="8" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F16" s="9"/>
     </row>
@@ -8087,11 +7838,11 @@
       <c r="A17" s="6"/>
       <c r="B17" s="2"/>
       <c r="C17" s="8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F17" s="9"/>
     </row>
@@ -8099,11 +7850,11 @@
       <c r="A18" s="6"/>
       <c r="B18" s="2"/>
       <c r="C18" s="8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D18" s="9"/>
       <c r="E18" s="8" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F18" s="9"/>
     </row>
@@ -8111,25 +7862,25 @@
       <c r="A19" s="6"/>
       <c r="B19" s="2"/>
       <c r="C19" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F19" s="9"/>
     </row>
     <row r="20" s="1" customFormat="1" spans="1:6">
       <c r="A20" s="6"/>
       <c r="B20" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F20" s="2"/>
     </row>
@@ -8137,11 +7888,11 @@
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F21" s="9"/>
     </row>
@@ -8149,13 +7900,13 @@
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="10" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F22" s="9"/>
     </row>
@@ -8164,10 +7915,10 @@
       <c r="B23" s="6"/>
       <c r="C23" s="11"/>
       <c r="D23" s="8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F23" s="9"/>
     </row>
@@ -8176,10 +7927,10 @@
       <c r="B24" s="6"/>
       <c r="C24" s="11"/>
       <c r="D24" s="8" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F24" s="16"/>
     </row>
@@ -8188,10 +7939,10 @@
       <c r="B25" s="6"/>
       <c r="C25" s="11"/>
       <c r="D25" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F25" s="9"/>
     </row>
@@ -8200,10 +7951,10 @@
       <c r="B26" s="6"/>
       <c r="C26" s="11"/>
       <c r="D26" s="8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F26" s="18"/>
     </row>
@@ -8212,10 +7963,10 @@
       <c r="B27" s="6"/>
       <c r="C27" s="11"/>
       <c r="D27" s="9" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F27" s="9"/>
     </row>
@@ -8224,10 +7975,10 @@
       <c r="B28" s="6"/>
       <c r="C28" s="11"/>
       <c r="D28" s="8" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F28" s="9"/>
     </row>
@@ -8236,10 +7987,10 @@
       <c r="B29" s="6"/>
       <c r="C29" s="11"/>
       <c r="D29" s="8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F29" s="9"/>
     </row>
@@ -8248,10 +7999,10 @@
       <c r="B30" s="6"/>
       <c r="C30" s="11"/>
       <c r="D30" s="8" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F30" s="9"/>
     </row>
@@ -8260,10 +8011,10 @@
       <c r="B31" s="6"/>
       <c r="C31" s="11"/>
       <c r="D31" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F31" s="9"/>
     </row>
@@ -8272,10 +8023,10 @@
       <c r="B32" s="6"/>
       <c r="C32" s="11"/>
       <c r="D32" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F32" s="9"/>
     </row>
@@ -8284,10 +8035,10 @@
       <c r="B33" s="6"/>
       <c r="C33" s="11"/>
       <c r="D33" s="8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F33" s="9"/>
     </row>
@@ -8296,7 +8047,7 @@
       <c r="B34" s="6"/>
       <c r="C34" s="11"/>
       <c r="D34" s="8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E34" s="17">
         <v>0.005</v>
@@ -8308,7 +8059,7 @@
       <c r="B35" s="6"/>
       <c r="C35" s="11"/>
       <c r="D35" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E35" s="17">
         <v>50</v>
@@ -8320,10 +8071,10 @@
       <c r="B36" s="6"/>
       <c r="C36" s="11"/>
       <c r="D36" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F36" s="18"/>
     </row>
@@ -8332,7 +8083,7 @@
       <c r="B37" s="6"/>
       <c r="C37" s="11"/>
       <c r="D37" s="8" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E37" s="17">
         <v>50</v>
@@ -8344,7 +8095,7 @@
       <c r="B38" s="6"/>
       <c r="C38" s="11"/>
       <c r="D38" s="8" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E38" s="17">
         <v>0.5</v>
@@ -8356,7 +8107,7 @@
       <c r="B39" s="6"/>
       <c r="C39" s="11"/>
       <c r="D39" s="8" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E39" s="17">
         <v>50</v>
@@ -8368,7 +8119,7 @@
       <c r="B40" s="6"/>
       <c r="C40" s="11"/>
       <c r="D40" s="8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E40" s="17">
         <v>0.5</v>
@@ -8380,10 +8131,10 @@
       <c r="B41" s="6"/>
       <c r="C41" s="11"/>
       <c r="D41" s="8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F41" s="9"/>
     </row>
@@ -8392,10 +8143,10 @@
       <c r="B42" s="6"/>
       <c r="C42" s="11"/>
       <c r="D42" s="8" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F42" s="9"/>
     </row>
@@ -8404,10 +8155,10 @@
       <c r="B43" s="6"/>
       <c r="C43" s="11"/>
       <c r="D43" s="8" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F43" s="9"/>
     </row>
@@ -8416,10 +8167,10 @@
       <c r="B44" s="6"/>
       <c r="C44" s="11"/>
       <c r="D44" s="8" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F44" s="9"/>
     </row>
@@ -8428,10 +8179,10 @@
       <c r="B45" s="6"/>
       <c r="C45" s="11"/>
       <c r="D45" s="8" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F45" s="9"/>
     </row>
@@ -8440,10 +8191,10 @@
       <c r="B46" s="6"/>
       <c r="C46" s="11"/>
       <c r="D46" s="8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F46" s="9"/>
     </row>
@@ -8452,10 +8203,10 @@
       <c r="B47" s="6"/>
       <c r="C47" s="11"/>
       <c r="D47" s="8" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F47" s="9"/>
     </row>
@@ -8464,10 +8215,10 @@
       <c r="B48" s="6"/>
       <c r="C48" s="11"/>
       <c r="D48" s="8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F48" s="9"/>
     </row>
@@ -8476,10 +8227,10 @@
       <c r="B49" s="6"/>
       <c r="C49" s="11"/>
       <c r="D49" s="8" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F49" s="9"/>
     </row>
@@ -8488,10 +8239,10 @@
       <c r="B50" s="6"/>
       <c r="C50" s="11"/>
       <c r="D50" s="8" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F50" s="9"/>
     </row>
@@ -8500,10 +8251,10 @@
       <c r="B51" s="6"/>
       <c r="C51" s="11"/>
       <c r="D51" s="8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F51" s="9"/>
     </row>
@@ -8512,10 +8263,10 @@
       <c r="B52" s="6"/>
       <c r="C52" s="11"/>
       <c r="D52" s="8" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F52" s="9"/>
     </row>
@@ -8524,10 +8275,10 @@
       <c r="B53" s="6"/>
       <c r="C53" s="11"/>
       <c r="D53" s="9" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F53" s="9"/>
     </row>
@@ -8536,13 +8287,13 @@
       <c r="B54" s="6"/>
       <c r="C54" s="11"/>
       <c r="D54" s="8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E54" s="19" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F54" s="19" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="55" s="1" customFormat="1" ht="34.5" customHeight="1" spans="1:6">
@@ -8550,10 +8301,10 @@
       <c r="B55" s="6"/>
       <c r="C55" s="11"/>
       <c r="D55" s="8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F55" s="9"/>
     </row>
@@ -8562,10 +8313,10 @@
       <c r="B56" s="6"/>
       <c r="C56" s="11"/>
       <c r="D56" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="F56" s="9"/>
     </row>
@@ -8574,10 +8325,10 @@
       <c r="B57" s="6"/>
       <c r="C57" s="12"/>
       <c r="D57" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F57" s="9"/>
     </row>

</xml_diff>